<commit_message>
fix: update default model to gemini-3.8-flash for Gemini API audio output
</commit_message>
<xml_diff>
--- a/Gemini_Voice_Studio_Lite_開発計画・仕様書.xlsx
+++ b/Gemini_Voice_Studio_Lite_開発計画・仕様書.xlsx
@@ -640,7 +640,7 @@
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Gemini 2.5 Flash / Gemini 2.0 Flash (Speech Generation対応)</t>
+          <t>Gemini 3.8 Flash / Gemini 3.0 Flash (Speech Generation対応)</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1206,7 @@
       </c>
       <c r="E5" s="11" t="inlineStr">
         <is>
-          <t>gemini-2.5-flash（初期値）, gemini-2.0-flash</t>
+          <t>gemini-3.8-flash（初期値）, gemini-3.0-flash</t>
         </is>
       </c>
     </row>

</xml_diff>